<commit_message>
Update estimation of possible detection (memory) with new messages size (add uid, type and up)
</commit_message>
<xml_diff>
--- a/docs/assets/images/User_description/Estimation of detection records on SD memory card.xlsx
+++ b/docs/assets/images/User_description/Estimation of detection records on SD memory card.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\btenaud\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\btenaud\Documents\02 - Projet Antenne-Terrier\02 - Git\rfid_m0.wiki\docs\assets\images\User_description\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -23,32 +23,8 @@
 </workbook>
 </file>
 
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>benjamin tenaud</author>
-  </authors>
-  <commentList>
-    <comment ref="C4" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">Size of controller format for 4GB : Pessimistic estimation for 2GB
-</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="41">
   <si>
     <t>Size [byte]</t>
   </si>
@@ -86,9 +62,6 @@
     <t>Vbat variation measurement [V]</t>
   </si>
   <si>
-    <t>Battery measurement data</t>
-  </si>
-  <si>
     <t>Max Vbat messages</t>
   </si>
   <si>
@@ -125,38 +98,62 @@
     <t>|- Duration if 1 tag / s</t>
   </si>
   <si>
-    <t>YYYY-MM-DD;HH:MM:SS.mmm;System; Start;</t>
-  </si>
-  <si>
-    <t>YYYY-MM-DD;HH:MM:SS.mmm;IR X;broken beam;</t>
-  </si>
-  <si>
-    <t>YYYY-MM-DD;HH:MM:SS.mmm;IR X;beam restored;</t>
-  </si>
-  <si>
-    <t>YYYY-MM-DD;HH:MM:SS.mmm;A0;250-229500045120;</t>
-  </si>
-  <si>
-    <t>YYYY-MM-DD;HH:MM:SS.mmm;Vbat;xx.xxV;</t>
-  </si>
-  <si>
-    <t>YYYY-MM-DD;HH:MM:SS.mmm;Shut Down Button;</t>
-  </si>
-  <si>
-    <t>YYYY-MM-DD;HH:MM:SS.mmm;System;RTC is ok;</t>
-  </si>
-  <si>
-    <t>Message *</t>
-  </si>
-  <si>
-    <t>* Pessimistic size with the more possible digits</t>
+    <t>Battery  data</t>
+  </si>
+  <si>
+    <t>Expected autonomy [day]</t>
+  </si>
+  <si>
+    <t>Max Up messages</t>
+  </si>
+  <si>
+    <t>Up</t>
+  </si>
+  <si>
+    <t>YYYY-MM-DD;HH:MM:SS.mmm;$uid_rfid_sensor$;inv_rfid_sensor;IR X;broken beam;</t>
+  </si>
+  <si>
+    <t>YYYY-MM-DD;HH:MM:SS.mmm;$uid_rfid_sensor$;inv_rfid_sensor;IR X;beam restored;</t>
+  </si>
+  <si>
+    <t>YYYY-MM-DD;HH:MM:SS.mmm;$uid_rfid_sensor$;inv_rfid_sensor;A0;250-229500045120;</t>
+  </si>
+  <si>
+    <t>YYYY-MM-DD;HH:MM:SS.mmm;$uid_mainboard$;inv_mainboard;System; Start;</t>
+  </si>
+  <si>
+    <t>YYYY-MM-DD;HH:MM:SS.mmm;$uid_mainboard$;inv_mainboard;System;RTC is ok;</t>
+  </si>
+  <si>
+    <t>YYYY-MM-DD;HH:MM:SS.mmm;$uid_mainboard$;inv_mainboard;Vbat;xx.xxV;</t>
+  </si>
+  <si>
+    <t>YYYY-MM-DD;HH:MM:SS.mmm;$uid_mainboard$;inv_mainboard;System;Up;</t>
+  </si>
+  <si>
+    <t>YYYY-MM-DD;HH:MM:SS.mmm;$uid_mainboard$;inv_mainboard;System;Shut Down Button;</t>
+  </si>
+  <si>
+    <t>Size of configuration file [byte] *</t>
+  </si>
+  <si>
+    <t>Size of assembly file [byte] *</t>
+  </si>
+  <si>
+    <t>* Large estimation for future options</t>
+  </si>
+  <si>
+    <t>Message **</t>
+  </si>
+  <si>
+    <t>** Pessimistic size with the more possible digits</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -194,12 +191,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="6">
@@ -294,7 +285,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -312,7 +303,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -346,10 +336,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -630,45 +628,45 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:I23"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="B2:I30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
-    <col min="2" max="2" width="48.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="83.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="21.7109375" customWidth="1"/>
-    <col min="4" max="4" width="14.5703125" customWidth="1"/>
-    <col min="5" max="5" width="16.28515625" customWidth="1"/>
-    <col min="6" max="6" width="28" customWidth="1"/>
-    <col min="7" max="7" width="15.28515625" customWidth="1"/>
+    <col min="4" max="4" width="11.7109375" customWidth="1"/>
+    <col min="5" max="5" width="12.28515625" customWidth="1"/>
+    <col min="6" max="6" width="36.5703125" customWidth="1"/>
+    <col min="7" max="7" width="17.5703125" customWidth="1"/>
     <col min="8" max="8" width="13.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B2" s="23" t="s">
+      <c r="B2" s="29" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="23"/>
-      <c r="F2" s="23" t="s">
-        <v>14</v>
-      </c>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
+      <c r="C2" s="29"/>
+      <c r="F2" s="29" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="13">
+      <c r="C3" s="12">
         <v>2</v>
       </c>
-      <c r="F3" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="G3" s="15" t="s">
+      <c r="F3" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="15" t="s">
+      <c r="H3" s="14" t="s">
         <v>0</v>
       </c>
     </row>
@@ -676,257 +674,314 @@
       <c r="B4" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="13">
-        <v>27994112</v>
+      <c r="C4" s="12">
+        <v>0</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G4" s="4">
         <v>1</v>
       </c>
       <c r="H4" s="4">
-        <f>G4*(C9+C10+$C$16*2)</f>
-        <v>83</v>
+        <f>G4*(C12+C13+$C$20*2)</f>
+        <v>143</v>
       </c>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="9">
+      <c r="C5" s="27">
         <f>C3*1000000000-C4</f>
-        <v>1972005888</v>
+        <v>2000000000</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G5" s="4">
         <v>1</v>
       </c>
       <c r="H5" s="4">
-        <f>G5*(C15+$C$16)</f>
-        <v>43</v>
+        <f>G5*(C19+$C$20)</f>
+        <v>80</v>
       </c>
     </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B6" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" s="7">
+        <v>512</v>
+      </c>
       <c r="F6" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" s="4">
+        <f>C28</f>
+        <v>20</v>
+      </c>
+      <c r="H6" s="4">
+        <f>G6*(C17+$C$20)</f>
+        <v>1360</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B7" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" s="2">
+        <v>512</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="G7" s="4">
+        <f>C30</f>
+        <v>480</v>
+      </c>
+      <c r="H7" s="4">
+        <f>G7*(C18+$C$20)</f>
+        <v>31680</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B8" s="28" t="s">
+        <v>38</v>
+      </c>
+      <c r="F8" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="G6" s="4">
-        <f>C23</f>
+      <c r="G8" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="H6" s="4">
-        <f>G6*(C14+$C$16)</f>
-        <v>760</v>
-      </c>
-    </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B7" s="23" t="s">
+      <c r="H8" s="4">
+        <f>C14*2+C15*2+C20*4</f>
+        <v>312</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="F9" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="H9" s="4">
+        <f>H8+C16+C20</f>
+        <v>392</v>
+      </c>
+    </row>
+    <row r="10" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B10" s="29" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="23"/>
-      <c r="F7" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="G7" s="11" t="s">
+      <c r="C10" s="29"/>
+    </row>
+    <row r="11" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B11" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="F11" s="29" t="s">
         <v>21</v>
       </c>
-      <c r="H7" s="4">
-        <f>C11*2+C12*2+C16*4</f>
-        <v>176</v>
-      </c>
-    </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B8" s="5" t="s">
+      <c r="G11" s="29"/>
+      <c r="H11" s="29"/>
+    </row>
+    <row r="12" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B12" s="26" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12" s="20">
+        <f>LEN(B12)</f>
+        <v>68</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="G12" s="7"/>
+      <c r="H12" s="17">
+        <f>C5-C6-C7-SUM(H4:H7)</f>
+        <v>1999965713</v>
+      </c>
+    </row>
+    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B13" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="C8" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="F8" s="3" t="s">
+      <c r="C13" s="20">
+        <f>LEN(B13)</f>
+        <v>71</v>
+      </c>
+      <c r="F13" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="G13" s="7"/>
+      <c r="H13" s="18">
+        <f>H12/H8</f>
+        <v>6410146.516025641</v>
+      </c>
+    </row>
+    <row r="14" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B14" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" s="20">
+        <f t="shared" ref="C14:C18" si="0">LEN(B14)</f>
+        <v>75</v>
+      </c>
+      <c r="F14" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="G14" s="7"/>
+      <c r="H14" s="17" t="str">
+        <f>INT(H13/3600/24) &amp; "j " &amp; INT((H13-INT(H13/3600/24)*24*3600)/3600) &amp; "h"</f>
+        <v>74j 4h</v>
+      </c>
+    </row>
+    <row r="15" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B15" s="26" t="s">
+        <v>29</v>
+      </c>
+      <c r="C15" s="20">
+        <f t="shared" si="0"/>
+        <v>77</v>
+      </c>
+      <c r="F15" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="G15" s="7"/>
+      <c r="H15" s="18">
+        <f>H12/H9</f>
+        <v>5101953.349489796</v>
+      </c>
+    </row>
+    <row r="16" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B16" s="26" t="s">
+        <v>30</v>
+      </c>
+      <c r="C16" s="20">
+        <f t="shared" si="0"/>
+        <v>78</v>
+      </c>
+      <c r="F16" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="G16" s="2"/>
+      <c r="H16" s="19" t="str">
+        <f>INT(H15/3600/24) &amp; "j " &amp; INT((H15-INT(H15/3600/24)*24*3600)/3600) &amp; "h"</f>
+        <v>59j 1h</v>
+      </c>
+    </row>
+    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B17" s="26" t="s">
+        <v>33</v>
+      </c>
+      <c r="C17" s="20">
+        <f t="shared" si="0"/>
+        <v>66</v>
+      </c>
+    </row>
+    <row r="18" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B18" s="26" t="s">
+        <v>34</v>
+      </c>
+      <c r="C18" s="20">
+        <f t="shared" si="0"/>
+        <v>64</v>
+      </c>
+    </row>
+    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B19" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="C19" s="20">
+        <f>LEN(B19)</f>
+        <v>78</v>
+      </c>
+    </row>
+    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B20" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C20" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B21" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="I21" s="22"/>
+    </row>
+    <row r="24" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B24" s="29" t="s">
+        <v>24</v>
+      </c>
+      <c r="C24" s="29"/>
+    </row>
+    <row r="25" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B25" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C25" s="8">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="26" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B26" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C26" s="8">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="27" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B27" t="s">
+        <v>11</v>
+      </c>
+      <c r="C27" s="11">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="28" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B28" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C28" s="24">
+        <f>(C25-C26)/C27</f>
         <v>20</v>
       </c>
-      <c r="G8" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="H8" s="4">
-        <f>H7+C13+C16</f>
-        <v>222</v>
-      </c>
-    </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B9" s="1" t="s">
+    </row>
+    <row r="29" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B29" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="21">
-        <f>LEN(B9)</f>
-        <v>38</v>
-      </c>
-    </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B10" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C10" s="21">
-        <f>LEN(B10)</f>
-        <v>41</v>
-      </c>
-    </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B11" s="1" t="s">
+      <c r="C29" s="11">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="30" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B30" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="C11" s="21">
-        <f t="shared" ref="C11:C15" si="0">LEN(B11)</f>
-        <v>41</v>
-      </c>
-      <c r="F11" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="G11" s="23"/>
-      <c r="H11" s="23"/>
-    </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B12" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="C12" s="21">
-        <f t="shared" si="0"/>
-        <v>43</v>
-      </c>
-      <c r="F12" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="G12" s="7"/>
-      <c r="H12" s="18">
-        <f>C5-SUM(H4:H6)</f>
-        <v>1972005002</v>
-      </c>
-    </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B13" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C13" s="21">
-        <f t="shared" si="0"/>
-        <v>44</v>
-      </c>
-      <c r="F13" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="G13" s="7"/>
-      <c r="H13" s="19">
-        <f>H12/H7</f>
-        <v>11204573.875</v>
-      </c>
-    </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B14" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C14" s="21">
-        <f t="shared" si="0"/>
-        <v>36</v>
-      </c>
-      <c r="F14" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="G14" s="7"/>
-      <c r="H14" s="18" t="str">
-        <f>INT(H13/3600/24) &amp; "j " &amp; INT((H13-INT(H13/3600/24)*24*3600)/3600) &amp; "h"</f>
-        <v>129j 16h</v>
-      </c>
-    </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B15" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C15" s="21">
-        <f t="shared" si="0"/>
-        <v>41</v>
-      </c>
-      <c r="F15" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="G15" s="7"/>
-      <c r="H15" s="19">
-        <f>H12/H8</f>
-        <v>8882905.4144144151</v>
-      </c>
-    </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B16" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C16" s="4">
-        <v>2</v>
-      </c>
-      <c r="F16" s="17" t="s">
-        <v>24</v>
-      </c>
-      <c r="G16" s="2"/>
-      <c r="H16" s="20" t="str">
-        <f>INT(H15/3600/24) &amp; "j " &amp; INT((H15-INT(H15/3600/24)*24*3600)/3600) &amp; "h"</f>
-        <v>102j 19h</v>
-      </c>
-    </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B17" s="22" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B19" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="C19" s="23"/>
-    </row>
-    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B20" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="C20" s="8">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B21" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="C21" s="8">
-        <v>12</v>
-      </c>
-      <c r="I21" s="24"/>
-    </row>
-    <row r="22" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B22" t="s">
-        <v>11</v>
-      </c>
-      <c r="C22" s="12">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="23" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B23" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C23" s="11">
-        <f>(C20-C21)/C22</f>
-        <v>20</v>
+      <c r="C30" s="10">
+        <f>C29*24</f>
+        <v>480</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B10:C10"/>
     <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B24:C24"/>
     <mergeCell ref="F2:H2"/>
     <mergeCell ref="F11:H11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>